<commit_message>
Vlookup and Hloolup index and matchs
</commit_message>
<xml_diff>
--- a/T388_Excel.xlsx
+++ b/T388_Excel.xlsx
@@ -8,14 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30ED5A1-8554-4E9D-8791-3C50885488E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D3DCB0-3088-46CA-B55D-1F93149D8A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{97914E35-3EC5-46A0-9D29-D522FBEA4F09}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97914E35-3EC5-46A0-9D29-D522FBEA4F09}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="50">
   <si>
     <t>ID</t>
   </si>
@@ -137,21 +135,6 @@
     <t>SHARE PRICE</t>
   </si>
   <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>Apr</t>
-  </si>
-  <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>July</t>
-  </si>
-  <si>
     <t>PRODUCT</t>
   </si>
   <si>
@@ -198,6 +181,9 @@
   </si>
   <si>
     <t>Vegetable</t>
+  </si>
+  <si>
+    <t>F21</t>
   </si>
 </sst>
 </file>
@@ -331,7 +317,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -350,10 +336,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -365,16 +348,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="15" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -691,17 +668,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB60FD70-39C4-4057-8347-98CA45557147}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FC74FB1-AD57-4850-AA87-E06A6A7A96BD}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:X32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -709,9 +677,12 @@
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -730,7 +701,7 @@
       <c r="F1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="9" t="s">
         <v>30</v>
       </c>
       <c r="I1" t="s">
@@ -739,8 +710,29 @@
       <c r="J1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="S1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="T1" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="W1" s="11">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -770,8 +762,29 @@
       <c r="J2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O2" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" s="11">
+        <v>40</v>
+      </c>
+      <c r="S2" s="11">
+        <v>2</v>
+      </c>
+      <c r="T2" s="11">
+        <v>80</v>
+      </c>
+      <c r="W2" s="11">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -801,8 +814,33 @@
       <c r="J3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O3" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" s="11">
+        <v>120</v>
+      </c>
+      <c r="S3" s="11">
+        <v>2</v>
+      </c>
+      <c r="T3" s="11">
+        <v>240</v>
+      </c>
+      <c r="W3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3">
+        <f>COUNTA(W1:W6)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -832,8 +870,33 @@
       <c r="J4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O4" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="R4" s="11">
+        <v>60</v>
+      </c>
+      <c r="S4" s="11">
+        <v>4</v>
+      </c>
+      <c r="T4" s="11">
+        <v>240</v>
+      </c>
+      <c r="W4" s="11">
+        <v>25</v>
+      </c>
+      <c r="X4">
+        <f>COUNTBLANK(W1:W6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -863,8 +926,29 @@
       <c r="J5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O5" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="R5" s="11">
+        <v>100</v>
+      </c>
+      <c r="S5" s="11">
+        <v>3</v>
+      </c>
+      <c r="T5" s="11">
+        <v>300</v>
+      </c>
+      <c r="W5" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -894,14 +978,53 @@
       <c r="J6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O6" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q6" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="R6" s="11">
+        <v>120</v>
+      </c>
+      <c r="S6" s="11">
+        <v>6</v>
+      </c>
+      <c r="T6" s="11">
+        <v>720</v>
+      </c>
+      <c r="W6" s="11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="O7" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P7" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q7" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="R7" s="11">
+        <v>25</v>
+      </c>
+      <c r="S7" s="11">
+        <v>2</v>
+      </c>
+      <c r="T7" s="11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="2" t="s">
@@ -910,14 +1033,14 @@
       <c r="D8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="3" t="s">
@@ -926,17 +1049,25 @@
       <c r="D9" s="1">
         <v>30</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="12">
         <v>46023</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="11">
         <v>205</v>
       </c>
       <c r="I9">
         <v>200</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="Q9">
+        <f>COUNTIF(Q2:Q7,"Fruit")</f>
+        <v>3</v>
+      </c>
+      <c r="R9">
+        <f>SUMIF(Q2:Q7,"Fruit",S2:S7)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="3" t="s">
@@ -945,14 +1076,22 @@
       <c r="D10" s="1">
         <v>45</v>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="12">
         <v>46054</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="11">
         <v>206.7</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="Q10">
+        <f>COUNTIFS(P2:P7,"Frozen",Q2:Q7,"vegetable")</f>
+        <v>2</v>
+      </c>
+      <c r="R10">
+        <f>SUMIFS(S2:S7,P2:P7,"Frozen",Q2:Q7,"Fruit")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="3" t="s">
@@ -961,14 +1100,18 @@
       <c r="D11" s="1">
         <v>44</v>
       </c>
-      <c r="F11" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="12">
-        <v>204.3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F11" s="12">
+        <v>46082</v>
+      </c>
+      <c r="G11" s="11">
+        <v>205</v>
+      </c>
+      <c r="K11">
+        <f>I9+I12</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="3" t="s">
@@ -977,43 +1120,37 @@
       <c r="D12" s="1">
         <v>15</v>
       </c>
-      <c r="F12" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="G12" s="12">
+      <c r="F12" s="12">
+        <v>46113</v>
+      </c>
+      <c r="G12" s="11">
         <v>207.1</v>
       </c>
       <c r="I12">
         <v>400</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="1">
         <v>45</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="12">
+      <c r="F13" s="12">
+        <v>46143</v>
+      </c>
+      <c r="G13" s="11">
         <v>208.1</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C14" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="9">
-        <v>25</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="G14" s="12">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F14" s="12">
+        <v>46174</v>
+      </c>
+      <c r="G14" s="11">
         <v>207.9</v>
       </c>
       <c r="K14">
@@ -1021,177 +1158,208 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="F15" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G15" s="12">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F15" s="12">
+        <v>46204</v>
+      </c>
+      <c r="G15" s="11">
         <v>208.2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="K16">
         <f>I12*6</f>
         <v>2400</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="I17">
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="K20">
         <f>I17+55</f>
         <v>1055</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="15" t="s">
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="B24" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="11">
         <v>40</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="E24" s="11">
+        <v>2</v>
+      </c>
+      <c r="F24" s="11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="11">
+        <v>120</v>
+      </c>
+      <c r="E25" s="11">
+        <v>2</v>
+      </c>
+      <c r="F25" s="11">
+        <v>240</v>
+      </c>
+      <c r="J25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="B26" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D26" s="11">
+        <v>60</v>
+      </c>
+      <c r="E26" s="11">
+        <v>4</v>
+      </c>
+      <c r="F26" s="11">
+        <v>240</v>
+      </c>
+      <c r="L26">
+        <f>J25+J27</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="B27" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" s="11">
+        <v>100</v>
+      </c>
+      <c r="E27" s="11">
+        <v>3</v>
+      </c>
+      <c r="F27" s="11">
+        <v>300</v>
+      </c>
+      <c r="J27">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+      <c r="B28" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="11">
+        <v>120</v>
+      </c>
+      <c r="E28" s="11">
+        <v>6</v>
+      </c>
+      <c r="F28" s="11">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B29" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="11">
+        <v>25</v>
+      </c>
+      <c r="E29" s="11">
+        <v>2</v>
+      </c>
+      <c r="F29" s="11">
         <v>50</v>
       </c>
-      <c r="C24" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D24" s="12">
-        <v>40</v>
-      </c>
-      <c r="E24" s="12">
-        <v>2</v>
-      </c>
-      <c r="F24" s="16">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="12">
-        <v>120</v>
-      </c>
-      <c r="E25" s="12">
-        <v>2</v>
-      </c>
-      <c r="F25" s="16">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="12">
-        <v>60</v>
-      </c>
-      <c r="E26" s="12">
-        <v>4</v>
-      </c>
-      <c r="F26" s="16">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27" s="12">
-        <v>100</v>
-      </c>
-      <c r="E27" s="12">
-        <v>3</v>
-      </c>
-      <c r="F27" s="16">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D28" s="12">
-        <v>120</v>
-      </c>
-      <c r="E28" s="12">
-        <v>6</v>
-      </c>
-      <c r="F28" s="16">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D29" s="12">
-        <v>25</v>
-      </c>
-      <c r="E29" s="12">
-        <v>2</v>
-      </c>
-      <c r="F29" s="16">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="12"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="11"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="11"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="D8:D14">
+  <conditionalFormatting sqref="D8:D13">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
@@ -1228,19 +1396,10 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D8:D14</xm:sqref>
+          <xm:sqref>D8:D13</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AB9FC98-78AE-4240-86AF-DAC89B581F95}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>